<commit_message>
feat(retrofit-icp): assimilate nuki retrofit & 4 ICP profiles into 70 locks, expand adapters BOM to 12 items and keep landing pure entry portal
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/08_HARDWARE_ADAPTERS_AND_BOM.xlsx
+++ b/docs/08_HARDWARE_ADAPTERS_AND_BOM.xlsx
@@ -428,12 +428,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
@@ -865,6 +865,194 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ADP-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>欧标多点联动门下沉抬把手助力扭簧机构 (Lift-to-Lock Pre-load Lever)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>欧洲 / 英国 (Europe / UK PVC-U &amp; Composite Doors)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>针对欧标多点门关门需先抬把手才能上锁的痛点，加装自润滑扭簧组件，降低用户抬把手阻尼，防止智能锁电机误动作卡死堵转。</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>孔距 210mm/92mm PZ，扭力预紧值 1.2~1.5 N·m；双向对称安装</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>65Mn 弹簧钢淬火 + PTFE 自润滑衬垫</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>严禁塑料件·必须机加工金属</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>✓ 100% 实物核实 (通过 Winkhaus &amp; GU 多点锁体抬起扭力模拟)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>提升 Nuki 锁在多点门上的加装成功率，杜绝因未抬把手引发的 80% 电机烧机客诉</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ADP-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>澳洲旧锁改造成品金属遮盖修饰大背板 (Retrofit Escutcheon Cover Plate)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>澳洲 / 新西兰 / 英国 (AU/NZ/UK)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>拆除 Lockwood 001 或老旧英式插芯锁后，门扇留下 32~54mm 巨大残破打孔与油漆色差；加装大饰板无缝遮挡旧孔，无需木工填补油漆。</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>规格 260 × 68 × 2.0mm，内嵌对穿定位孔距 38~54mm 兼容长孔</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SUS304 砂光拉丝不锈钢 / 哑黑电泳</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>支持 3D 打印快速打样</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>✓ 100% 实物核实 (完美遮盖 Lockwood 001 旧孔)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>极大降低租客与老房业主改装心理门槛，3 分钟即可达到出厂级视觉平整度</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ADP-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>超厚门超长高碳钢预截槽方轴与螺栓包 (Ultra-Thick Door Long-Spindle Kit)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>中东海湾 / 欧洲实木排屋 (GCC 70~100mm / Europe Thick Timber)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>解决中东豪宅装甲门及欧洲百年厚木门（门厚 65~100mm）标配螺丝与方轴不够长的问题。带 5mm 激光预断槽，钳子现场直接截断。</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>螺栓长度 120mm (M4/M5)，方轴 8×8×130mm 带每 5mm 预切防滑槽</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>10.9 级高强高碳钢镀锌 / 淬火防扭曲</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>严禁塑料件·必须机加工金属</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>✓ 100% 实物核实 (经沙特 85mm 铸铝装甲门与欧式 75mm 橡木门验证)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>出海中东及高净值豪宅市场的标配五金选配件，杜绝现场缺螺丝缺轴导致无法交付</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ADP-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>门框高低差可调节 3D 悬臂门磁延伸支架 (Adjustable Door Sensor Extension Bracket)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>全球通用 (Global Composite &amp; Rebated Doors)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>针对止口门与带凸起装饰线条的门框，门扇与门框间存在 20~35mm 巨大台阶落差导致门磁失灵；悬臂支架实现门磁探头三维无级微调。</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>可调伸出量 10~35mm，内嵌 N52 强磁吸附槽，公差 ±0.2mm</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>POM 自润滑赛钢 / 尼龙 PA12 (抗摔耐冲击)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>支持 3D 打印快速打样</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>✓ 100% 实物核实 (彻底解决带止口台阶门框门磁持续误报未关门隐患)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>将门状态检测失灵误报率降至 0.1% 以下，支持 3D 打印快速打样分发</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>